<commit_message>
updated gcode and notes
</commit_message>
<xml_diff>
--- a/Prusa Work/Adhesion Testing/Optimization Testing/Optimal Design Runs.xlsx
+++ b/Prusa Work/Adhesion Testing/Optimization Testing/Optimal Design Runs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github Stuff\Cylindrical-4th-Axis-Printer\Prusa Work\Adhesion Testing\Optimization Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{509537DA-C726-4059-BDFF-D442AEB42B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FA73F4-6FB5-4748-AEB4-D1421FBE265E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6" yWindow="6" windowWidth="23028" windowHeight="12228" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>Run</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>From Variance Testing</t>
+  </si>
+  <si>
+    <t>Shaft collar failed on ADMET, sample must be repeated</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -142,13 +148,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FBC1B571-4B51-41CD-ADCE-1AB837F4C666}" name="Table4" displayName="Table4" ref="B2:K104" totalsRowShown="0">
-  <autoFilter ref="B2:K104" xr:uid="{FBC1B571-4B51-41CD-ADCE-1AB837F4C666}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="5"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B2:K104" xr:uid="{FBC1B571-4B51-41CD-ADCE-1AB837F4C666}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9C86E860-61AA-4FEE-8EB4-A30E954E2ABD}" name="Run" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{A20EC31A-F218-4399-BC4B-A51A407258CC}" name="Mandrel"/>
@@ -475,7 +475,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B3">
         <v>1</v>
       </c>
@@ -504,7 +504,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B4">
         <v>1</v>
       </c>
@@ -530,7 +530,7 @@
         <v>73.643699999999995</v>
       </c>
     </row>
-    <row r="5" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B5">
         <v>1</v>
       </c>
@@ -556,7 +556,7 @@
         <v>89.305999999999997</v>
       </c>
     </row>
-    <row r="6" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B6">
         <v>1</v>
       </c>
@@ -582,7 +582,7 @@
         <v>73.695700000000002</v>
       </c>
     </row>
-    <row r="7" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B7">
         <v>1</v>
       </c>
@@ -608,7 +608,7 @@
         <v>48.312100000000001</v>
       </c>
     </row>
-    <row r="8" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B8">
         <v>1</v>
       </c>
@@ -634,7 +634,7 @@
         <v>85.577500000000001</v>
       </c>
     </row>
-    <row r="9" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B9">
         <v>2</v>
       </c>
@@ -663,7 +663,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B10">
         <v>2</v>
       </c>
@@ -689,7 +689,7 @@
         <v>100.43049999999999</v>
       </c>
     </row>
-    <row r="11" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B11">
         <v>2</v>
       </c>
@@ -715,7 +715,7 @@
         <v>90.388499999999993</v>
       </c>
     </row>
-    <row r="12" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B12">
         <v>2</v>
       </c>
@@ -741,7 +741,7 @@
         <v>101.8031</v>
       </c>
     </row>
-    <row r="13" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B13">
         <v>2</v>
       </c>
@@ -767,7 +767,7 @@
         <v>62.641399999999997</v>
       </c>
     </row>
-    <row r="14" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B14">
         <v>2</v>
       </c>
@@ -793,7 +793,7 @@
         <v>72.420699999999997</v>
       </c>
     </row>
-    <row r="15" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B15">
         <v>3</v>
       </c>
@@ -822,7 +822,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="2:11" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.55000000000000004">
       <c r="B16">
         <v>3</v>
       </c>
@@ -848,7 +848,7 @@
         <v>85.453800000000001</v>
       </c>
     </row>
-    <row r="17" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B17">
         <v>3</v>
       </c>
@@ -874,7 +874,7 @@
         <v>82.852099999999993</v>
       </c>
     </row>
-    <row r="18" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B18">
         <v>3</v>
       </c>
@@ -900,7 +900,7 @@
         <v>103.39100000000001</v>
       </c>
     </row>
-    <row r="19" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B19">
         <v>3</v>
       </c>
@@ -926,7 +926,7 @@
         <v>59.873199999999997</v>
       </c>
     </row>
-    <row r="20" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B20">
         <v>3</v>
       </c>
@@ -952,7 +952,7 @@
         <v>63.8598</v>
       </c>
     </row>
-    <row r="21" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B21">
         <v>4</v>
       </c>
@@ -975,7 +975,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B22">
         <v>4</v>
       </c>
@@ -998,7 +998,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B23">
         <v>4</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="24" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B24">
         <v>4</v>
       </c>
@@ -1044,7 +1044,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="25" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B25">
         <v>4</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="2:9" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.55000000000000004">
       <c r="B26">
         <v>4</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="33" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B33">
         <v>6</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="34" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B34">
         <v>6</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B35">
         <v>6</v>
       </c>
@@ -1297,7 +1297,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="36" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B36">
         <v>6</v>
       </c>
@@ -1320,7 +1320,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="37" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B37">
         <v>6</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B38">
         <v>6</v>
       </c>
@@ -1366,7 +1366,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B39">
         <v>7</v>
       </c>
@@ -1388,8 +1388,11 @@
       <c r="H39">
         <v>2</v>
       </c>
-    </row>
-    <row r="40" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="J39" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B40">
         <v>7</v>
       </c>
@@ -1411,8 +1414,11 @@
       <c r="H40">
         <v>2</v>
       </c>
-    </row>
-    <row r="41" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="J40" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B41">
         <v>7</v>
       </c>
@@ -1435,7 +1441,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="42" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B42">
         <v>7</v>
       </c>
@@ -1458,7 +1464,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="43" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B43">
         <v>7</v>
       </c>
@@ -1481,7 +1487,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="44" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B44">
         <v>7</v>
       </c>
@@ -1504,7 +1510,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="45" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B45">
         <v>8</v>
       </c>
@@ -1527,7 +1533,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="46" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B46">
         <v>8</v>
       </c>
@@ -1550,7 +1556,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="47" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B47">
         <v>8</v>
       </c>
@@ -1573,7 +1579,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="48" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="2:10" x14ac:dyDescent="0.55000000000000004">
       <c r="B48">
         <v>8</v>
       </c>
@@ -1596,7 +1602,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="49" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B49">
         <v>8</v>
       </c>
@@ -1619,7 +1625,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="50" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B50">
         <v>8</v>
       </c>
@@ -1642,7 +1648,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="51" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B51">
         <v>9</v>
       </c>
@@ -1665,7 +1671,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="52" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B52">
         <v>9</v>
       </c>
@@ -1688,7 +1694,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="53" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B53">
         <v>9</v>
       </c>
@@ -1711,7 +1717,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="54" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B54">
         <v>9</v>
       </c>
@@ -1734,7 +1740,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="55" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B55">
         <v>9</v>
       </c>
@@ -1757,7 +1763,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B56">
         <v>9</v>
       </c>
@@ -1780,7 +1786,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="57" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B57">
         <v>10</v>
       </c>
@@ -1803,7 +1809,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="58" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B58">
         <v>10</v>
       </c>
@@ -1826,7 +1832,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="59" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B59">
         <v>10</v>
       </c>
@@ -1849,7 +1855,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="60" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B60">
         <v>10</v>
       </c>
@@ -1872,7 +1878,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="61" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B61">
         <v>10</v>
       </c>
@@ -1895,7 +1901,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="62" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B62">
         <v>10</v>
       </c>
@@ -1918,7 +1924,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="63" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B63">
         <v>11</v>
       </c>
@@ -1941,7 +1947,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B64">
         <v>11</v>
       </c>
@@ -1964,7 +1970,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="65" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B65">
         <v>11</v>
       </c>
@@ -1987,7 +1993,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="66" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B66">
         <v>11</v>
       </c>
@@ -2010,7 +2016,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="67" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="67" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B67">
         <v>11</v>
       </c>
@@ -2033,7 +2039,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="68" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="68" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B68">
         <v>11</v>
       </c>
@@ -2056,7 +2062,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="69" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B69">
         <v>12</v>
       </c>
@@ -2079,7 +2085,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="70" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="70" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B70">
         <v>12</v>
       </c>
@@ -2102,7 +2108,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="71" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="71" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B71">
         <v>12</v>
       </c>
@@ -2125,7 +2131,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="72" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B72">
         <v>12</v>
       </c>
@@ -2148,7 +2154,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="73" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B73">
         <v>12</v>
       </c>
@@ -2171,7 +2177,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="74" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="74" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B74">
         <v>12</v>
       </c>
@@ -2194,7 +2200,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="75" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B75">
         <v>13</v>
       </c>
@@ -2217,7 +2223,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="76" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B76">
         <v>13</v>
       </c>
@@ -2240,7 +2246,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="77" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B77">
         <v>13</v>
       </c>
@@ -2263,7 +2269,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="78" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="78" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B78">
         <v>13</v>
       </c>
@@ -2286,7 +2292,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="79" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B79">
         <v>13</v>
       </c>
@@ -2309,7 +2315,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="80" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="80" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B80">
         <v>13</v>
       </c>
@@ -2332,7 +2338,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="81" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B81">
         <v>14</v>
       </c>
@@ -2355,7 +2361,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="82" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="82" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B82">
         <v>14</v>
       </c>
@@ -2378,7 +2384,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="83" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B83">
         <v>14</v>
       </c>
@@ -2401,7 +2407,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="84" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B84">
         <v>14</v>
       </c>
@@ -2424,7 +2430,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="85" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="85" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B85">
         <v>14</v>
       </c>
@@ -2447,7 +2453,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="86" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="86" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B86">
         <v>14</v>
       </c>
@@ -2470,7 +2476,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="87" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="87" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B87">
         <v>15</v>
       </c>
@@ -2493,7 +2499,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="88" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B88">
         <v>15</v>
       </c>
@@ -2516,7 +2522,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="89" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="89" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B89">
         <v>15</v>
       </c>
@@ -2539,7 +2545,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="90" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="90" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B90">
         <v>15</v>
       </c>
@@ -2562,7 +2568,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="91" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B91">
         <v>15</v>
       </c>
@@ -2585,7 +2591,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="92" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="92" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B92">
         <v>15</v>
       </c>
@@ -2608,7 +2614,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="93" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="93" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B93" s="1">
         <v>16</v>
       </c>
@@ -2631,7 +2637,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="94" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="94" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B94" s="1">
         <v>16</v>
       </c>
@@ -2654,7 +2660,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="95" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B95" s="1">
         <v>16</v>
       </c>
@@ -2677,7 +2683,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="96" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B96" s="1">
         <v>16</v>
       </c>
@@ -2700,7 +2706,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="97" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="97" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B97" s="1">
         <v>16</v>
       </c>
@@ -2723,7 +2729,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="98" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="98" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B98" s="1">
         <v>16</v>
       </c>
@@ -2746,7 +2752,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="99" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="99" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B99" s="1">
         <v>17</v>
       </c>
@@ -2769,7 +2775,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="100" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="100" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B100" s="1">
         <v>17</v>
       </c>
@@ -2792,7 +2798,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="101" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="101" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B101" s="1">
         <v>17</v>
       </c>
@@ -2815,7 +2821,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="102" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="102" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B102" s="1">
         <v>17</v>
       </c>
@@ -2838,7 +2844,7 @@
         <v>1.75</v>
       </c>
     </row>
-    <row r="103" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="103" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B103" s="1">
         <v>17</v>
       </c>
@@ -2861,7 +2867,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="104" spans="2:8" hidden="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="104" spans="2:8" x14ac:dyDescent="0.55000000000000004">
       <c r="B104" s="1">
         <v>17</v>
       </c>

</xml_diff>